<commit_message>
feat: add order payment tracking and WhatsApp confirmation totals
</commit_message>
<xml_diff>
--- a/artifacts/admin-orders/export-fixture.xlsx
+++ b/artifacts/admin-orders/export-fixture.xlsx
@@ -11,7 +11,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
-    <col min="1" max="18" width="24" customWidth="1"/>
+    <col min="1" max="20" width="24" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -105,6 +105,16 @@
           <t xml:space="preserve">Internal ID</t>
         </is>
       </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Payment received (INR)</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Remaining amount (INR)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -195,16 +205,22 @@
           <t xml:space="preserve">order-id</t>
         </is>
       </c>
+      <c r="S2" t="n">
+        <v>234.5</v>
+      </c>
+      <c r="T2" t="n">
+        <v>1000</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R2"/>
+  <autoFilter ref="A1:T2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
-    <col min="1" max="18" width="24" customWidth="1"/>
+    <col min="1" max="20" width="24" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>